<commit_message>
Update 8416 and add 534ez submission tracking
</commit_message>
<xml_diff>
--- a/strategy/bio/post-go-live/21p-8416/21P-8416 Post-Go-Live Submission Tracker.xlsx
+++ b/strategy/bio/post-go-live/21p-8416/21P-8416 Post-Go-Live Submission Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VBAHOUASHIOM\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE6E2F43-C656-4EFB-BB9D-5AE692BB83F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A08BC3D-5C5F-45BC-A44A-E2CD67699295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{AF2C844A-C5C8-460C-A4FB-B4FB01059A32}"/>
+    <workbookView xWindow="-2663" yWindow="-10882" windowWidth="19365" windowHeight="10244" xr2:uid="{AF2C844A-C5C8-460C-A4FB-B4FB01059A32}"/>
   </bookViews>
   <sheets>
     <sheet name="21P-8416" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>UUID</t>
   </si>
@@ -96,6 +96,21 @@
   </si>
   <si>
     <t>21P-8416 Post-Go-Live Submission Tracker</t>
+  </si>
+  <si>
+    <t>f56e9f01-5f40-45ab-8f3e-d9fb0afa68d4</t>
+  </si>
+  <si>
+    <t>517026de-80c7-461f-bfb0-52886e859519</t>
+  </si>
+  <si>
+    <t>469f79a8-955c-446f-9180-e5f25dd9012c</t>
+  </si>
+  <si>
+    <t>480198a0-5ff8-4a64-ac79-ea9dddca26b5</t>
+  </si>
+  <si>
+    <t>ee7cf9e6-13e4-41c7-b385-fb544b4903a2</t>
   </si>
 </sst>
 </file>
@@ -965,7 +980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{693FDA50-AF9A-4F34-A5D2-8EFB6209C293}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40.1796875" customWidth="1"/>
@@ -997,11 +1012,11 @@
         <v>8</v>
       </c>
       <c r="B4">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C4" s="4">
         <f>B4/B3</f>
-        <v>0.10714285714285714</v>
+        <v>0.16666666666666666</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -1133,6 +1148,61 @@
       </c>
       <c r="C16" s="1">
         <v>46056</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="1">
+        <v>46065</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="1">
+        <v>46068</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="1">
+        <v>46069</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="1">
+        <v>46070</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="1">
+        <v>46070</v>
       </c>
     </row>
   </sheetData>

</xml_diff>